<commit_message>
Atualiza notas 2C Manha 2º Bimestre
</commit_message>
<xml_diff>
--- a/sources/2C_Manha_2_Bimestre.xlsx
+++ b/sources/2C_Manha_2_Bimestre.xlsx
@@ -61,7 +61,7 @@
     <x:t>Conselho Segundo Bimestre</x:t>
   </x:si>
   <x:si>
-    <x:t>237</x:t>
+    <x:t>307</x:t>
   </x:si>
   <x:si>
     <x:t>0 (Soma de todas as eletivas)</x:t>
@@ -183,387 +183,384 @@
     <x:t>100%</x:t>
   </x:si>
   <x:si>
+    <x:t>97%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARTHUR ISAAC SANTOS TEOFILO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ativo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>80%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>83%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRENO ADRIANO GONCALVES DE ASSIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>90%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>92%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CARLA YASMIM GALDINO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>89%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>91%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DIOGO JANUARIO DIAS DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>75%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>79%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EDUARDO FAUSTINO EVANGELISTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>17</x:t>
+  </x:si>
+  <x:si>
+    <x:t>59%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>64%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKENE AKONOBI MONTEIRO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>74%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FELIPE ARIEL PEREIRA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Não Comparecimento</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16</x:t>
+  </x:si>
+  <x:si>
+    <x:t>18</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>32</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>37%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>53%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FELIPE OLIVEIRA DE SOUZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>68%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>77%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FERNANDA FERREIRA LOPES FONSECA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Baixa - Transferência</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GABRIEL CORREIA DOS SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Transferido</x:t>
+  </x:si>
+  <x:si>
+    <x:t>86%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GABRIELLE LUIZA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>84%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEOVANA SALES VILELLA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEOVANNA PEREIRA SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GIOVANNA LOPES FERREIRA DOS SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>93%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUSTAVO LEONCIO INDALICIO DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>72%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>76%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HERSON ALDO ROQUE HUANCA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>98%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IVAN JHONNY MURILLO MENDOZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JOAO HENRIQUE BICIATTO MARTINS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>71%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAREN MAYSA CONDORI MAYTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>95%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAUAN HENRIQUE SOUZA COSTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAWAN SANTANA SOUZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>81%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>85%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAYKY FELICIANO DE ASSIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>78%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KEVIN ANDERSON SANTOS SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRIS MARC TRACY GEORGE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>65%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LARISSA SANTANA DA COSTA DIAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>34</x:t>
+  </x:si>
+  <x:si>
+    <x:t>36</x:t>
+  </x:si>
+  <x:si>
+    <x:t>36%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>99%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LEANDRO VINICIUS DIAS MAURO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>88%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LIVIA KETLINN FEITOZA DE SA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MANUELA ERNESTO DOS SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MELANIE HANNA GOMEZ CABRERA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>69%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>73%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MICKAEL RODRIGUES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>82%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>94%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MIGUEL PEREIRA DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PEDIRA FRANCISCA YALA SOKIKA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PEDRO HENRIQUE RODRIGUES BORDIGNON</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PEDRO HENRIQUE SOUZA BOMBARDA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PEDRO TOMAS JOÃO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RAFAELA SANTIAGO DE MORAES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RAFAELY ARAUJO QUÉRCIA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>87%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RAQUEL CRISTINA SOUZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RICHARD CANUTO ALCIDES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RICKELME CINTRA DE SANTANA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>24</x:t>
+  </x:si>
+  <x:si>
+    <x:t>43%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>61%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RODRIGO DA SILVA ARAUJO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>28</x:t>
+  </x:si>
+  <x:si>
+    <x:t>26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>47%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAMUEL DOS SANTOS LINS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VITÓRIA PEREIRA DE ALMEIDA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WANDERLEY APPOLINARIO JUNIOR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WELLINGTON REIS FERREIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YASMIN SILVA DE OLIVEIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YASMIN VITORIA FARIAS PEDREIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LIVIA MARIA ALY MATHIAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BEATRIZ VITORIA COSTA DOS SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ANDREY MENEZES SANTOS</x:t>
+  </x:si>
+  <x:si>
     <x:t>96%</x:t>
   </x:si>
   <x:si>
-    <x:t>ARTHUR ISAAC SANTOS TEOFILO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ativo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8</x:t>
-  </x:si>
-  <x:si>
-    <x:t>80%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>82%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRENO ADRIANO GONCALVES DE ASSIS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>88%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>91%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CARLA YASMIM GALDINO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9</x:t>
-  </x:si>
-  <x:si>
-    <x:t>90%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DIOGO JANUARIO DIAS DA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>13</x:t>
-  </x:si>
-  <x:si>
-    <x:t>72%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>78%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EDUARDO FAUSTINO EVANGELISTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>58%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>64%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKENE AKONOBI MONTEIRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>17</x:t>
-  </x:si>
-  <x:si>
-    <x:t>70%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>83%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FELIPE ARIEL PEREIRA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Não Comparecimento</x:t>
-  </x:si>
-  <x:si>
-    <x:t>16</x:t>
-  </x:si>
-  <x:si>
-    <x:t>18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>30</x:t>
-  </x:si>
-  <x:si>
-    <x:t>14</x:t>
-  </x:si>
-  <x:si>
-    <x:t>37%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>55%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FELIPE OLIVEIRA DE SOUZA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>19</x:t>
-  </x:si>
-  <x:si>
-    <x:t>67%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FERNANDA FERREIRA LOPES FONSECA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Baixa - Transferência</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GABRIEL CORREIA DOS SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Transferido</x:t>
-  </x:si>
-  <x:si>
-    <x:t>86%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>75%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GABRIELLE LUIZA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEOVANA SALES VILELLA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEOVANNA PEREIRA SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>74%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GIOVANNA LOPES FERREIRA DOS SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>92%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUSTAVO LEONCIO INDALICIO DA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>76%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HERSON ALDO ROQUE HUANCA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>94%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IVAN JHONNY MURILLO MENDOZA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>97%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JOAO HENRIQUE BICIATTO MARTINS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>68%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAREN MAYSA CONDORI MAYTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAUAN HENRIQUE SOUZA COSTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>73%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAWAN SANTANA SOUZA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAYKY FELICIANO DE ASSIS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>85%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KEVIN ANDERSON SANTOS SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>69%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRIS MARC TRACY GEORGE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>66%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>79%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LARISSA SANTANA DA COSTA DIAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>34</x:t>
-  </x:si>
-  <x:si>
-    <x:t>36</x:t>
-  </x:si>
-  <x:si>
-    <x:t>36%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>102%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LEANDRO VINICIUS DIAS MAURO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>87%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>93%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LIVIA KETLINN FEITOZA DE SA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MANUELA ERNESTO DOS SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>89%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>95%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MELANIE HANNA GOMEZ CABRERA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>65%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MICKAEL RODRIGUES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MIGUEL PEREIRA DA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>81%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PEDIRA FRANCISCA YALA SOKIKA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>99%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PEDRO HENRIQUE RODRIGUES BORDIGNON</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PEDRO HENRIQUE SOUZA BOMBARDA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PEDRO TOMAS JOÃO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RAFAELA SANTIAGO DE MORAES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RAFAELY ARAUJO QUÉRCIA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RAQUEL CRISTINA SOUZA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RICHARD CANUTO ALCIDES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RICKELME CINTRA DE SANTANA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>43%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>63%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RODRIGO DA SILVA ARAUJO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>28</x:t>
-  </x:si>
-  <x:si>
-    <x:t>41%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>47%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SAMUEL DOS SANTOS LINS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VITÓRIA PEREIRA DE ALMEIDA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WANDERLEY APPOLINARIO JUNIOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WELLINGTON REIS FERREIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YASMIN SILVA DE OLIVEIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>77%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YASMIN VITORIA FARIAS PEDREIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LIVIA MARIA ALY MATHIAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BEATRIZ VITORIA COSTA DOS SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANDREY MENEZES SANTOS</x:t>
-  </x:si>
-  <x:si>
     <x:t>GABRIEL DOS SANTOS LANÇA</x:t>
   </x:si>
   <x:si>
     <x:t>VINICIUS PEREIRA DOS SANTOS</x:t>
   </x:si>
   <x:si>
-    <x:t>84%</x:t>
-  </x:si>
-  <x:si>
     <x:t>ISADORA REDUA RONDINONE</x:t>
   </x:si>
   <x:si>
     <x:t>MATHEUS MARRONE SALDANHA CABRAL</x:t>
   </x:si>
   <x:si>
-    <x:t>98%</x:t>
-  </x:si>
-  <x:si>
     <x:t>JOSÉ FRANCISCO FERREIRA DE LIMA</x:t>
   </x:si>
   <x:si>
@@ -586,6 +583,9 @@
   </x:si>
   <x:si>
     <x:t>Aulas Dadas: 42</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Aulas Dadas: 50</x:t>
   </x:si>
   <x:si>
     <x:t>Legenda</x:t>
@@ -1635,10 +1635,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO13" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP13" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ13" s="12">
         <x:v>1</x:v>
@@ -1647,10 +1647,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS13" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT13" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU13" s="12">
         <x:v>1</x:v>
@@ -1820,25 +1820,25 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AN14" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO14" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AP14" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ14" s="12">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AR14" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS14" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AT14" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU14" s="12">
         <x:v>2</x:v>
@@ -1877,13 +1877,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG14" s="12">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="BH14" s="12" t="s">
         <x:v>61</x:v>
       </x:c>
       <x:c r="BI14" s="12">
-        <x:v>96</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="BJ14" s="12" t="s">
         <x:v>62</x:v>
@@ -2008,25 +2008,25 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="AN15" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO15" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AP15" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ15" s="12">
         <x:v>3</x:v>
       </x:c>
       <x:c r="AR15" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS15" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT15" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU15" s="12">
         <x:v>3</x:v>
@@ -2065,13 +2065,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG15" s="12">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="BH15" s="12" t="s">
         <x:v>65</x:v>
       </x:c>
       <x:c r="BI15" s="12">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="BJ15" s="12" t="s">
         <x:v>66</x:v>
@@ -2196,25 +2196,25 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AN16" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AO16" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP16" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ16" s="12">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AR16" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS16" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AT16" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU16" s="12">
         <x:v>4</x:v>
@@ -2253,21 +2253,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG16" s="12">
-        <x:v>23</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="BH16" s="12" t="s">
         <x:v>69</x:v>
       </x:c>
       <x:c r="BI16" s="12">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="BJ16" s="12" t="s">
-        <x:v>66</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:62">
       <x:c r="A17" s="11" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B17" s="12" t="s">
         <x:v>53</x:v>
@@ -2330,7 +2330,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="V17" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="W17" s="12">
         <x:v>5</x:v>
@@ -2375,7 +2375,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AK17" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="AL17" s="12" t="s">
         <x:v>49</x:v>
@@ -2384,25 +2384,25 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AN17" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO17" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="AP17" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ17" s="12">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AR17" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS17" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT17" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU17" s="12">
         <x:v>5</x:v>
@@ -2432,7 +2432,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="BD17" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE17" s="12" t="s">
         <x:v>60</x:v>
@@ -2441,21 +2441,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG17" s="12">
-        <x:v>66</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="BH17" s="12" t="s">
-        <x:v>73</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="BI17" s="12">
-        <x:v>119</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="BJ17" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:62">
       <x:c r="A18" s="11" t="s">
-        <x:v>75</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B18" s="12" t="s">
         <x:v>53</x:v>
@@ -2539,7 +2539,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AC18" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AD18" s="12" t="s">
         <x:v>49</x:v>
@@ -2563,7 +2563,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AK18" s="12" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="AL18" s="12" t="s">
         <x:v>49</x:v>
@@ -2572,25 +2572,25 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="AN18" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO18" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="AP18" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ18" s="12">
         <x:v>6</x:v>
       </x:c>
       <x:c r="AR18" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS18" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AT18" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU18" s="12">
         <x:v>6</x:v>
@@ -2599,7 +2599,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AW18" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AX18" s="12" t="s">
         <x:v>49</x:v>
@@ -2629,21 +2629,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG18" s="12">
-        <x:v>100</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="BH18" s="12" t="s">
-        <x:v>78</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="BI18" s="12">
-        <x:v>198</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="BJ18" s="12" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:62">
       <x:c r="A19" s="11" t="s">
-        <x:v>80</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B19" s="12" t="s">
         <x:v>53</x:v>
@@ -2712,7 +2712,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="X19" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="Y19" s="12" t="s">
         <x:v>64</x:v>
@@ -2742,7 +2742,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="AH19" s="12" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="AI19" s="12">
         <x:v>7</x:v>
@@ -2760,25 +2760,25 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="AN19" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AO19" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP19" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ19" s="12">
         <x:v>7</x:v>
       </x:c>
       <x:c r="AR19" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS19" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AT19" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU19" s="12">
         <x:v>7</x:v>
@@ -2799,7 +2799,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="BA19" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="BB19" s="12" t="s">
         <x:v>49</x:v>
@@ -2808,7 +2808,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="BD19" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE19" s="12" t="s">
         <x:v>60</x:v>
@@ -2817,33 +2817,33 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG19" s="12">
-        <x:v>71</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="BH19" s="12" t="s">
-        <x:v>82</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="BI19" s="12">
-        <x:v>92</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="BJ19" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:62">
       <x:c r="A20" s="11" t="s">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B20" s="12" t="s">
-        <x:v>85</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C20" s="12">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D20" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E20" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="F20" s="12" t="s">
         <x:v>49</x:v>
@@ -2855,7 +2855,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="I20" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="J20" s="12" t="s">
         <x:v>49</x:v>
@@ -2888,7 +2888,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="T20" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="U20" s="12" t="s">
         <x:v>59</x:v>
@@ -2924,10 +2924,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="AF20" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AG20" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AH20" s="12" t="s">
         <x:v>49</x:v>
@@ -2939,7 +2939,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AK20" s="12" t="s">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="AL20" s="12" t="s">
         <x:v>49</x:v>
@@ -2951,10 +2951,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO20" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="AP20" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ20" s="12">
         <x:v>8</x:v>
@@ -2963,19 +2963,19 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS20" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="AT20" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU20" s="12">
         <x:v>8</x:v>
       </x:c>
       <x:c r="AV20" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AW20" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AX20" s="12" t="s">
         <x:v>49</x:v>
@@ -2987,7 +2987,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="BA20" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="BB20" s="12" t="s">
         <x:v>49</x:v>
@@ -3005,21 +3005,21 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="BG20" s="12">
-        <x:v>150</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="BH20" s="12" t="s">
-        <x:v>90</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="BI20" s="12">
-        <x:v>236</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="BJ20" s="12" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:62">
       <x:c r="A21" s="11" t="s">
-        <x:v>92</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B21" s="12" t="s">
         <x:v>53</x:v>
@@ -3127,7 +3127,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="AK21" s="12" t="s">
-        <x:v>93</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="AL21" s="12" t="s">
         <x:v>49</x:v>
@@ -3136,25 +3136,25 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="AN21" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO21" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AP21" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ21" s="12">
         <x:v>9</x:v>
       </x:c>
       <x:c r="AR21" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS21" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AT21" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU21" s="12">
         <x:v>9</x:v>
@@ -3184,33 +3184,33 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="BD21" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE21" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="BF21" s="12" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG21" s="12">
-        <x:v>78</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="BH21" s="12" t="s">
-        <x:v>94</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="BI21" s="12">
-        <x:v>120</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="BJ21" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:62">
       <x:c r="A22" s="11" t="s">
-        <x:v>95</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B22" s="12" t="s">
-        <x:v>96</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C22" s="12">
         <x:v>10</x:v>
@@ -3327,10 +3327,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO22" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP22" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ22" s="12">
         <x:v>10</x:v>
@@ -3339,10 +3339,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS22" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT22" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU22" s="12">
         <x:v>10</x:v>
@@ -3390,15 +3390,15 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="BJ22" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:62">
       <x:c r="A23" s="11" t="s">
-        <x:v>97</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B23" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C23" s="12">
         <x:v>11</x:v>
@@ -3515,10 +3515,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO23" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP23" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ23" s="12">
         <x:v>11</x:v>
@@ -3527,10 +3527,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS23" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AT23" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU23" s="12">
         <x:v>11</x:v>
@@ -3569,21 +3569,21 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="BG23" s="12">
-        <x:v>32</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="BH23" s="12" t="s">
-        <x:v>99</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="BI23" s="12">
-        <x:v>129</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="BJ23" s="12" t="s">
-        <x:v>100</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:62">
       <x:c r="A24" s="11" t="s">
-        <x:v>101</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B24" s="12" t="s">
         <x:v>53</x:v>
@@ -3646,7 +3646,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="V24" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="W24" s="12">
         <x:v>12</x:v>
@@ -3700,25 +3700,25 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="AN24" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO24" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP24" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ24" s="12">
         <x:v>12</x:v>
       </x:c>
       <x:c r="AR24" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS24" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT24" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU24" s="12">
         <x:v>12</x:v>
@@ -3757,24 +3757,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG24" s="12">
-        <x:v>42</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="BH24" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="BI24" s="12">
-        <x:v>79</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="BJ24" s="12" t="s">
-        <x:v>99</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:62">
       <x:c r="A25" s="11" t="s">
-        <x:v>102</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B25" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C25" s="12">
         <x:v>13</x:v>
@@ -3891,10 +3891,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO25" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP25" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ25" s="12">
         <x:v>13</x:v>
@@ -3903,10 +3903,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS25" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT25" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU25" s="12">
         <x:v>13</x:v>
@@ -3959,10 +3959,10 @@
     </x:row>
     <x:row r="26" spans="1:62">
       <x:c r="A26" s="11" t="s">
-        <x:v>103</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B26" s="12" t="s">
-        <x:v>96</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C26" s="12">
         <x:v>14</x:v>
@@ -4079,10 +4079,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO26" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP26" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ26" s="12">
         <x:v>14</x:v>
@@ -4091,10 +4091,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS26" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT26" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU26" s="12">
         <x:v>14</x:v>
@@ -4142,15 +4142,15 @@
         <x:v>139</x:v>
       </x:c>
       <x:c r="BJ26" s="12" t="s">
-        <x:v>104</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:62">
       <x:c r="A27" s="11" t="s">
-        <x:v>105</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B27" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C27" s="12">
         <x:v>15</x:v>
@@ -4267,10 +4267,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO27" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP27" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ27" s="12">
         <x:v>15</x:v>
@@ -4279,10 +4279,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS27" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT27" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU27" s="12">
         <x:v>15</x:v>
@@ -4330,12 +4330,12 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="BJ27" s="12" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:62">
       <x:c r="A28" s="11" t="s">
-        <x:v>107</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B28" s="12" t="s">
         <x:v>53</x:v>
@@ -4359,7 +4359,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="I28" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="J28" s="12" t="s">
         <x:v>49</x:v>
@@ -4443,7 +4443,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AK28" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AL28" s="12" t="s">
         <x:v>49</x:v>
@@ -4452,25 +4452,25 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="AN28" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO28" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="AP28" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ28" s="12">
         <x:v>16</x:v>
       </x:c>
       <x:c r="AR28" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS28" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT28" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU28" s="12">
         <x:v>16</x:v>
@@ -4479,7 +4479,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="AW28" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AX28" s="12" t="s">
         <x:v>49</x:v>
@@ -4509,21 +4509,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG28" s="12">
-        <x:v>72</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="BH28" s="12" t="s">
-        <x:v>82</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="BI28" s="12">
-        <x:v>134</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="BJ28" s="12" t="s">
-        <x:v>108</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:62">
       <x:c r="A29" s="11" t="s">
-        <x:v>109</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B29" s="12" t="s">
         <x:v>53</x:v>
@@ -4559,7 +4559,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="M29" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="N29" s="12" t="s">
         <x:v>64</x:v>
@@ -4604,7 +4604,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="AB29" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AC29" s="12" t="s">
         <x:v>49</x:v>
@@ -4634,31 +4634,31 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="AL29" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="AM29" s="12">
         <x:v>17</x:v>
       </x:c>
       <x:c r="AN29" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO29" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AP29" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ29" s="12">
         <x:v>17</x:v>
       </x:c>
       <x:c r="AR29" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS29" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT29" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU29" s="12">
         <x:v>17</x:v>
@@ -4697,21 +4697,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG29" s="12">
-        <x:v>15</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="BH29" s="12" t="s">
-        <x:v>110</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="BI29" s="12">
-        <x:v>2</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="BJ29" s="12" t="s">
-        <x:v>50</x:v>
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:62">
       <x:c r="A30" s="11" t="s">
-        <x:v>111</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B30" s="12" t="s">
         <x:v>53</x:v>
@@ -4828,13 +4828,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="AN30" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO30" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AP30" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ30" s="12">
         <x:v>18</x:v>
@@ -4843,10 +4843,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS30" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT30" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU30" s="12">
         <x:v>18</x:v>
@@ -4885,21 +4885,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG30" s="12">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="BH30" s="12" t="s">
-        <x:v>112</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="BI30" s="12">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="BJ30" s="12" t="s">
-        <x:v>112</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:62">
       <x:c r="A31" s="11" t="s">
-        <x:v>113</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="B31" s="12" t="s">
         <x:v>53</x:v>
@@ -4962,7 +4962,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="V31" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="W31" s="12">
         <x:v>19</x:v>
@@ -5007,7 +5007,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="AK31" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AL31" s="12" t="s">
         <x:v>49</x:v>
@@ -5016,25 +5016,25 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="AN31" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AO31" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AP31" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ31" s="12">
         <x:v>19</x:v>
       </x:c>
       <x:c r="AR31" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS31" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AT31" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU31" s="12">
         <x:v>19</x:v>
@@ -5073,21 +5073,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG31" s="12">
-        <x:v>77</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="BH31" s="12" t="s">
-        <x:v>114</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="BI31" s="12">
-        <x:v>156</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="BJ31" s="12" t="s">
-        <x:v>73</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:62">
       <x:c r="A32" s="11" t="s">
-        <x:v>115</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B32" s="12" t="s">
         <x:v>47</x:v>
@@ -5207,10 +5207,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO32" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP32" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ32" s="12">
         <x:v>20</x:v>
@@ -5219,10 +5219,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS32" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT32" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU32" s="12">
         <x:v>20</x:v>
@@ -5270,15 +5270,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="BJ32" s="12" t="s">
-        <x:v>110</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:62">
       <x:c r="A33" s="11" t="s">
-        <x:v>116</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B33" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C33" s="12">
         <x:v>21</x:v>
@@ -5383,7 +5383,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AK33" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AL33" s="12" t="s">
         <x:v>49</x:v>
@@ -5395,10 +5395,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO33" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AP33" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ33" s="12">
         <x:v>21</x:v>
@@ -5407,10 +5407,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS33" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AT33" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU33" s="12">
         <x:v>21</x:v>
@@ -5449,24 +5449,24 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="BG33" s="12">
-        <x:v>63</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="BH33" s="12" t="s">
-        <x:v>117</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="BI33" s="12">
-        <x:v>125</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="BJ33" s="12" t="s">
-        <x:v>108</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:62">
       <x:c r="A34" s="11" t="s">
-        <x:v>118</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B34" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C34" s="12">
         <x:v>22</x:v>
@@ -5583,10 +5583,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO34" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP34" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ34" s="12">
         <x:v>22</x:v>
@@ -5595,10 +5595,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS34" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AT34" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU34" s="12">
         <x:v>22</x:v>
@@ -5637,21 +5637,21 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="BG34" s="12">
-        <x:v>47</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="BH34" s="12" t="s">
-        <x:v>61</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="BI34" s="12">
-        <x:v>75</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="BJ34" s="12" t="s">
-        <x:v>99</x:v>
+        <x:v>122</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:62">
       <x:c r="A35" s="11" t="s">
-        <x:v>119</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="B35" s="12" t="s">
         <x:v>53</x:v>
@@ -5714,7 +5714,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="V35" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="W35" s="12">
         <x:v>23</x:v>
@@ -5768,25 +5768,25 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="AN35" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AO35" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AP35" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ35" s="12">
         <x:v>23</x:v>
       </x:c>
       <x:c r="AR35" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS35" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT35" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU35" s="12">
         <x:v>23</x:v>
@@ -5825,21 +5825,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG35" s="12">
-        <x:v>58</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="BH35" s="12" t="s">
-        <x:v>108</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="BI35" s="12">
-        <x:v>81</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="BJ35" s="12" t="s">
-        <x:v>120</x:v>
+        <x:v>122</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:62">
       <x:c r="A36" s="11" t="s">
-        <x:v>121</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B36" s="12" t="s">
         <x:v>53</x:v>
@@ -5956,25 +5956,25 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="AN36" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO36" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AP36" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ36" s="12">
         <x:v>24</x:v>
       </x:c>
       <x:c r="AR36" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS36" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AT36" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU36" s="12">
         <x:v>24</x:v>
@@ -6004,7 +6004,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="BD36" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE36" s="12" t="s">
         <x:v>59</x:v>
@@ -6013,21 +6013,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG36" s="12">
-        <x:v>74</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="BH36" s="12" t="s">
-        <x:v>122</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="BI36" s="12">
-        <x:v>140</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="BJ36" s="12" t="s">
-        <x:v>104</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:62">
       <x:c r="A37" s="11" t="s">
-        <x:v>123</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="B37" s="12" t="s">
         <x:v>53</x:v>
@@ -6051,7 +6051,7 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="I37" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="J37" s="12" t="s">
         <x:v>49</x:v>
@@ -6135,7 +6135,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AK37" s="12" t="s">
-        <x:v>124</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="AL37" s="12" t="s">
         <x:v>49</x:v>
@@ -6144,25 +6144,25 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="AN37" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AO37" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="AP37" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ37" s="12">
         <x:v>25</x:v>
       </x:c>
       <x:c r="AR37" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS37" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AT37" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU37" s="12">
         <x:v>25</x:v>
@@ -6171,7 +6171,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AW37" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AX37" s="12" t="s">
         <x:v>49</x:v>
@@ -6192,7 +6192,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="BD37" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE37" s="12" t="s">
         <x:v>56</x:v>
@@ -6201,21 +6201,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG37" s="12">
-        <x:v>80</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BH37" s="12" t="s">
-        <x:v>125</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="BI37" s="12">
-        <x:v>115</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="BJ37" s="12" t="s">
-        <x:v>126</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:62">
       <x:c r="A38" s="11" t="s">
-        <x:v>127</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B38" s="12" t="s">
         <x:v>53</x:v>
@@ -6230,7 +6230,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="F38" s="12" t="s">
-        <x:v>128</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="G38" s="12">
         <x:v>26</x:v>
@@ -6239,10 +6239,10 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="I38" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="J38" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="K38" s="12">
         <x:v>26</x:v>
@@ -6278,7 +6278,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="V38" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="W38" s="12">
         <x:v>26</x:v>
@@ -6299,7 +6299,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AC38" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AD38" s="12" t="s">
         <x:v>49</x:v>
@@ -6311,10 +6311,10 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AG38" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AH38" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AI38" s="12">
         <x:v>26</x:v>
@@ -6323,34 +6323,34 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AK38" s="12" t="s">
-        <x:v>129</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="AL38" s="12" t="s">
-        <x:v>129</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="AM38" s="12">
         <x:v>26</x:v>
       </x:c>
       <x:c r="AN38" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO38" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="AP38" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="AQ38" s="12">
         <x:v>26</x:v>
       </x:c>
       <x:c r="AR38" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS38" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AT38" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU38" s="12">
         <x:v>26</x:v>
@@ -6359,10 +6359,10 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AW38" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="AX38" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="AY38" s="12">
         <x:v>26</x:v>
@@ -6371,10 +6371,10 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="BA38" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="BB38" s="12" t="s">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="BC38" s="12">
         <x:v>26</x:v>
@@ -6383,27 +6383,27 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="BE38" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="BF38" s="12" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG38" s="12">
-        <x:v>151</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="BH38" s="12" t="s">
-        <x:v>131</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="BI38" s="12">
-        <x:v>-10</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="BJ38" s="12" t="s">
-        <x:v>132</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:62">
       <x:c r="A39" s="11" t="s">
-        <x:v>133</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B39" s="12" t="s">
         <x:v>53</x:v>
@@ -6520,25 +6520,25 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="AN39" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO39" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP39" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ39" s="12">
         <x:v>27</x:v>
       </x:c>
       <x:c r="AR39" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS39" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT39" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU39" s="12">
         <x:v>27</x:v>
@@ -6577,21 +6577,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG39" s="12">
-        <x:v>30</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="BH39" s="12" t="s">
-        <x:v>134</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="BI39" s="12">
-        <x:v>38</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="BJ39" s="12" t="s">
-        <x:v>135</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:62">
       <x:c r="A40" s="11" t="s">
-        <x:v>136</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B40" s="12" t="s">
         <x:v>53</x:v>
@@ -6708,25 +6708,25 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="AN40" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AO40" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP40" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ40" s="12">
         <x:v>28</x:v>
       </x:c>
       <x:c r="AR40" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS40" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AT40" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU40" s="12">
         <x:v>28</x:v>
@@ -6765,21 +6765,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG40" s="12">
-        <x:v>41</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="BH40" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="BI40" s="12">
-        <x:v>77</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="BJ40" s="12" t="s">
-        <x:v>99</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:62">
       <x:c r="A41" s="11" t="s">
-        <x:v>137</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B41" s="12" t="s">
         <x:v>53</x:v>
@@ -6896,25 +6896,25 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="AN41" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AO41" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AP41" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ41" s="12">
         <x:v>29</x:v>
       </x:c>
       <x:c r="AR41" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS41" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT41" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU41" s="12">
         <x:v>29</x:v>
@@ -6953,21 +6953,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG41" s="12">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="BH41" s="12" t="s">
-        <x:v>138</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BI41" s="12">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="BJ41" s="12" t="s">
-        <x:v>139</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:62">
       <x:c r="A42" s="11" t="s">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B42" s="12" t="s">
         <x:v>53</x:v>
@@ -7084,25 +7084,25 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="AN42" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO42" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AP42" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ42" s="12">
         <x:v>30</x:v>
       </x:c>
       <x:c r="AR42" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS42" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AT42" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU42" s="12">
         <x:v>30</x:v>
@@ -7135,22 +7135,22 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="BE42" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="BF42" s="12" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG42" s="12">
-        <x:v>82</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="BH42" s="12" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="BI42" s="12">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="BJ42" s="12" t="s">
         <x:v>141</x:v>
-      </x:c>
-      <x:c r="BI42" s="12">
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="BJ42" s="12" t="s">
-        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:62">
@@ -7191,7 +7191,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="M43" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="N43" s="12" t="s">
         <x:v>64</x:v>
@@ -7263,34 +7263,34 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="AK43" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AL43" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AM43" s="12">
         <x:v>31</x:v>
       </x:c>
       <x:c r="AN43" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AO43" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="AP43" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ43" s="12">
         <x:v>31</x:v>
       </x:c>
       <x:c r="AR43" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS43" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT43" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU43" s="12">
         <x:v>31</x:v>
@@ -7329,21 +7329,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG43" s="12">
-        <x:v>41</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="BH43" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="BI43" s="12">
-        <x:v>22</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="BJ43" s="12" t="s">
-        <x:v>51</x:v>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:62">
       <x:c r="A44" s="11" t="s">
-        <x:v>143</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B44" s="12" t="s">
         <x:v>53</x:v>
@@ -7451,34 +7451,34 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AK44" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AL44" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="AM44" s="12">
         <x:v>32</x:v>
       </x:c>
       <x:c r="AN44" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO44" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="AP44" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ44" s="12">
         <x:v>32</x:v>
       </x:c>
       <x:c r="AR44" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS44" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AT44" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU44" s="12">
         <x:v>32</x:v>
@@ -7511,27 +7511,27 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="BE44" s="12" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="BF44" s="12" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="BG44" s="12">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="BH44" s="12" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="BF44" s="12" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="BG44" s="12">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="BH44" s="12" t="s">
-        <x:v>144</x:v>
-      </x:c>
       <x:c r="BI44" s="12">
-        <x:v>36</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="BJ44" s="12" t="s">
-        <x:v>135</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:62">
       <x:c r="A45" s="11" t="s">
-        <x:v>145</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B45" s="12" t="s">
         <x:v>53</x:v>
@@ -7648,25 +7648,25 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AN45" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AO45" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP45" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ45" s="12">
         <x:v>33</x:v>
       </x:c>
       <x:c r="AR45" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS45" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT45" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU45" s="12">
         <x:v>33</x:v>
@@ -7714,7 +7714,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="BJ45" s="12" t="s">
-        <x:v>146</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:62">
@@ -7755,7 +7755,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="M46" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="N46" s="12" t="s">
         <x:v>49</x:v>
@@ -7836,25 +7836,25 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="AN46" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO46" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AP46" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ46" s="12">
         <x:v>34</x:v>
       </x:c>
       <x:c r="AR46" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS46" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT46" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU46" s="12">
         <x:v>34</x:v>
@@ -7893,16 +7893,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG46" s="12">
-        <x:v>23</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="BH46" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="BI46" s="12">
-        <x:v>40</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="BJ46" s="12" t="s">
-        <x:v>135</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:62">
@@ -8027,10 +8027,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO47" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP47" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ47" s="12">
         <x:v>35</x:v>
@@ -8039,10 +8039,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS47" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT47" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU47" s="12">
         <x:v>35</x:v>
@@ -8090,7 +8090,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="BJ47" s="12" t="s">
-        <x:v>146</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:62">
@@ -8212,25 +8212,25 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="AN48" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AO48" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AP48" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ48" s="12">
         <x:v>36</x:v>
       </x:c>
       <x:c r="AR48" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS48" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AT48" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU48" s="12">
         <x:v>36</x:v>
@@ -8269,16 +8269,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG48" s="12">
-        <x:v>28</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="BH48" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="BI48" s="12">
-        <x:v>46</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="BJ48" s="12" t="s">
-        <x:v>106</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:62">
@@ -8403,10 +8403,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO49" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP49" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ49" s="12">
         <x:v>37</x:v>
@@ -8415,10 +8415,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS49" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT49" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU49" s="12">
         <x:v>37</x:v>
@@ -8466,7 +8466,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="BJ49" s="12" t="s">
-        <x:v>146</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:62">
@@ -8507,7 +8507,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="M50" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="N50" s="12" t="s">
         <x:v>49</x:v>
@@ -8588,25 +8588,25 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="AN50" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AO50" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AP50" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ50" s="12">
         <x:v>38</x:v>
       </x:c>
       <x:c r="AR50" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS50" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT50" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU50" s="12">
         <x:v>38</x:v>
@@ -8645,21 +8645,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG50" s="12">
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="BH50" s="12" t="s">
         <x:v>65</x:v>
       </x:c>
       <x:c r="BI50" s="12">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BJ50" s="12" t="s">
-        <x:v>99</x:v>
+        <x:v>152</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:62">
       <x:c r="A51" s="11" t="s">
-        <x:v>152</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B51" s="12" t="s">
         <x:v>53</x:v>
@@ -8767,7 +8767,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AK51" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AL51" s="12" t="s">
         <x:v>49</x:v>
@@ -8776,25 +8776,25 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="AN51" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AO51" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AP51" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ51" s="12">
         <x:v>39</x:v>
       </x:c>
       <x:c r="AR51" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS51" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT51" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU51" s="12">
         <x:v>39</x:v>
@@ -8824,30 +8824,30 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="BD51" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE51" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="BF51" s="12" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG51" s="12">
-        <x:v>67</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BH51" s="12" t="s">
-        <x:v>73</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="BI51" s="12">
-        <x:v>101</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="BJ51" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:62">
       <x:c r="A52" s="11" t="s">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B52" s="12" t="s">
         <x:v>53</x:v>
@@ -8964,25 +8964,25 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="AN52" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO52" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AP52" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ52" s="12">
         <x:v>40</x:v>
       </x:c>
       <x:c r="AR52" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS52" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT52" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU52" s="12">
         <x:v>40</x:v>
@@ -9021,21 +9021,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG52" s="12">
-        <x:v>14</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="BH52" s="12" t="s">
-        <x:v>110</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="BI52" s="12">
-        <x:v>17</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="BJ52" s="12" t="s">
-        <x:v>112</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:62">
       <x:c r="A53" s="11" t="s">
-        <x:v>154</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B53" s="12" t="s">
         <x:v>53</x:v>
@@ -9059,7 +9059,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="I53" s="12" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="J53" s="12" t="s">
         <x:v>49</x:v>
@@ -9107,7 +9107,7 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="Y53" s="12" t="s">
-        <x:v>128</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="Z53" s="12" t="s">
         <x:v>49</x:v>
@@ -9131,7 +9131,7 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="AG53" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AH53" s="12" t="s">
         <x:v>49</x:v>
@@ -9143,7 +9143,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AK53" s="12" t="s">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="AL53" s="12" t="s">
         <x:v>49</x:v>
@@ -9152,25 +9152,25 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="AN53" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO53" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="AP53" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ53" s="12">
         <x:v>41</x:v>
       </x:c>
       <x:c r="AR53" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS53" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AT53" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU53" s="12">
         <x:v>41</x:v>
@@ -9200,7 +9200,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="BD53" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE53" s="12" t="s">
         <x:v>60</x:v>
@@ -9209,21 +9209,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG53" s="12">
-        <x:v>136</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="BH53" s="12" t="s">
-        <x:v>155</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="BI53" s="12">
-        <x:v>201</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="BJ53" s="12" t="s">
-        <x:v>156</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:62">
       <x:c r="A54" s="11" t="s">
-        <x:v>157</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B54" s="12" t="s">
         <x:v>53</x:v>
@@ -9238,7 +9238,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="F54" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="G54" s="12">
         <x:v>42</x:v>
@@ -9247,7 +9247,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="I54" s="12" t="s">
-        <x:v>93</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="J54" s="12" t="s">
         <x:v>49</x:v>
@@ -9307,7 +9307,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AC54" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="AD54" s="12" t="s">
         <x:v>49</x:v>
@@ -9319,7 +9319,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="AG54" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="AH54" s="12" t="s">
         <x:v>49</x:v>
@@ -9331,7 +9331,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AK54" s="12" t="s">
-        <x:v>158</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="AL54" s="12" t="s">
         <x:v>49</x:v>
@@ -9340,25 +9340,25 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="AN54" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO54" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="AP54" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ54" s="12">
         <x:v>42</x:v>
       </x:c>
       <x:c r="AR54" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS54" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AT54" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU54" s="12">
         <x:v>42</x:v>
@@ -9367,7 +9367,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="AW54" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AX54" s="12" t="s">
         <x:v>49</x:v>
@@ -9397,21 +9397,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG54" s="12">
-        <x:v>140</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="BH54" s="12" t="s">
-        <x:v>159</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="BI54" s="12">
-        <x:v>291</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="BJ54" s="12" t="s">
-        <x:v>160</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:62">
       <x:c r="A55" s="11" t="s">
-        <x:v>161</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B55" s="12" t="s">
         <x:v>53</x:v>
@@ -9528,25 +9528,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="AN55" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AO55" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AP55" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ55" s="12">
         <x:v>43</x:v>
       </x:c>
       <x:c r="AR55" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS55" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT55" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU55" s="12">
         <x:v>43</x:v>
@@ -9585,24 +9585,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG55" s="12">
-        <x:v>25</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="BH55" s="12" t="s">
-        <x:v>138</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="BI55" s="12">
-        <x:v>40</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="BJ55" s="12" t="s">
-        <x:v>135</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:62">
       <x:c r="A56" s="11" t="s">
-        <x:v>162</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B56" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C56" s="12">
         <x:v>44</x:v>
@@ -9719,10 +9719,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO56" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP56" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ56" s="12">
         <x:v>44</x:v>
@@ -9731,10 +9731,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS56" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT56" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU56" s="12">
         <x:v>44</x:v>
@@ -9782,12 +9782,12 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="BJ56" s="12" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:62">
       <x:c r="A57" s="11" t="s">
-        <x:v>163</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B57" s="12" t="s">
         <x:v>53</x:v>
@@ -9904,25 +9904,25 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="AN57" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO57" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP57" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ57" s="12">
         <x:v>45</x:v>
       </x:c>
       <x:c r="AR57" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS57" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT57" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU57" s="12">
         <x:v>45</x:v>
@@ -9952,7 +9952,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="BD57" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE57" s="12" t="s">
         <x:v>56</x:v>
@@ -9964,18 +9964,18 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="BH57" s="12" t="s">
-        <x:v>138</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="BI57" s="12">
         <x:v>53</x:v>
       </x:c>
       <x:c r="BJ57" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:62">
       <x:c r="A58" s="11" t="s">
-        <x:v>164</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B58" s="12" t="s">
         <x:v>53</x:v>
@@ -10083,34 +10083,34 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AK58" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AL58" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="AM58" s="12">
         <x:v>46</x:v>
       </x:c>
       <x:c r="AN58" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO58" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AP58" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ58" s="12">
         <x:v>46</x:v>
       </x:c>
       <x:c r="AR58" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS58" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT58" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU58" s="12">
         <x:v>46</x:v>
@@ -10149,21 +10149,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG58" s="12">
-        <x:v>46</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="BH58" s="12" t="s">
-        <x:v>144</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="BI58" s="12">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="BJ58" s="12" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:62">
       <x:c r="A59" s="11" t="s">
-        <x:v>165</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B59" s="12" t="s">
         <x:v>53</x:v>
@@ -10232,7 +10232,7 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="X59" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="Y59" s="12" t="s">
         <x:v>58</x:v>
@@ -10271,7 +10271,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="AK59" s="12" t="s">
-        <x:v>166</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="AL59" s="12" t="s">
         <x:v>49</x:v>
@@ -10280,25 +10280,25 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="AN59" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AO59" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AP59" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ59" s="12">
         <x:v>47</x:v>
       </x:c>
       <x:c r="AR59" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS59" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AT59" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU59" s="12">
         <x:v>47</x:v>
@@ -10337,16 +10337,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG59" s="12">
-        <x:v>54</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="BH59" s="12" t="s">
-        <x:v>167</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="BI59" s="12">
-        <x:v>95</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BJ59" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:62">
@@ -10468,25 +10468,25 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AN60" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AO60" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AP60" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ60" s="12">
         <x:v>48</x:v>
       </x:c>
       <x:c r="AR60" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS60" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT60" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU60" s="12">
         <x:v>48</x:v>
@@ -10516,7 +10516,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="BD60" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE60" s="12" t="s">
         <x:v>56</x:v>
@@ -10525,16 +10525,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG60" s="12">
-        <x:v>49</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="BH60" s="12" t="s">
-        <x:v>126</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="BI60" s="12">
-        <x:v>107</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="BJ60" s="12" t="s">
-        <x:v>61</x:v>
+        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:62">
@@ -10563,7 +10563,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="I61" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="J61" s="12" t="s">
         <x:v>49</x:v>
@@ -10611,7 +10611,7 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="Y61" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="Z61" s="12" t="s">
         <x:v>49</x:v>
@@ -10647,7 +10647,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="AK61" s="12" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="AL61" s="12" t="s">
         <x:v>49</x:v>
@@ -10656,25 +10656,25 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="AN61" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO61" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="AP61" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ61" s="12">
         <x:v>49</x:v>
       </x:c>
       <x:c r="AR61" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AS61" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT61" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU61" s="12">
         <x:v>49</x:v>
@@ -10704,7 +10704,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BD61" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE61" s="12" t="s">
         <x:v>60</x:v>
@@ -10713,16 +10713,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG61" s="12">
-        <x:v>80</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="BH61" s="12" t="s">
-        <x:v>125</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="BI61" s="12">
-        <x:v>99</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="BJ61" s="12" t="s">
-        <x:v>62</x:v>
+        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:62">
@@ -10808,7 +10808,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="AB62" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AC62" s="12" t="s">
         <x:v>49</x:v>
@@ -10844,25 +10844,25 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="AN62" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AO62" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="AP62" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ62" s="12">
         <x:v>50</x:v>
       </x:c>
       <x:c r="AR62" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS62" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT62" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU62" s="12">
         <x:v>50</x:v>
@@ -10901,16 +10901,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG62" s="12">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="BH62" s="12" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="BI62" s="12">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="BH62" s="12" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="BI62" s="12">
-        <x:v>22</x:v>
-      </x:c>
       <x:c r="BJ62" s="12" t="s">
-        <x:v>51</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:62">
@@ -10987,7 +10987,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="Y63" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="Z63" s="12" t="s">
         <x:v>49</x:v>
@@ -10996,7 +10996,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="AB63" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="AC63" s="12" t="s">
         <x:v>49</x:v>
@@ -11032,25 +11032,25 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="AN63" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO63" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AP63" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ63" s="12">
         <x:v>51</x:v>
       </x:c>
       <x:c r="AR63" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS63" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT63" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU63" s="12">
         <x:v>51</x:v>
@@ -11089,21 +11089,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG63" s="12">
-        <x:v>7</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="BH63" s="12" t="s">
-        <x:v>112</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="BI63" s="12">
-        <x:v>5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="BJ63" s="12" t="s">
-        <x:v>146</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:62">
       <x:c r="A64" s="11" t="s">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B64" s="12" t="s">
         <x:v>53</x:v>
@@ -11127,7 +11127,7 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="I64" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="J64" s="12" t="s">
         <x:v>49</x:v>
@@ -11220,13 +11220,13 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="AN64" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO64" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="AP64" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ64" s="12">
         <x:v>52</x:v>
@@ -11235,10 +11235,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS64" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AT64" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU64" s="12">
         <x:v>52</x:v>
@@ -11277,21 +11277,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG64" s="12">
-        <x:v>71</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="BH64" s="12" t="s">
-        <x:v>82</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="BI64" s="12">
-        <x:v>71</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="BJ64" s="12" t="s">
-        <x:v>61</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="65" spans="1:62">
       <x:c r="A65" s="11" t="s">
-        <x:v>173</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B65" s="12" t="s">
         <x:v>53</x:v>
@@ -11408,25 +11408,25 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AN65" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO65" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AP65" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ65" s="12">
         <x:v>53</x:v>
       </x:c>
       <x:c r="AR65" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS65" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT65" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU65" s="12">
         <x:v>53</x:v>
@@ -11465,16 +11465,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG65" s="12">
-        <x:v>38</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="BH65" s="12" t="s">
-        <x:v>174</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="BI65" s="12">
-        <x:v>38</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="BJ65" s="12" t="s">
-        <x:v>174</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="66" spans="1:62">
@@ -11599,10 +11599,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO66" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AP66" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ66" s="12">
         <x:v>54</x:v>
@@ -11611,10 +11611,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS66" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AT66" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU66" s="12">
         <x:v>54</x:v>
@@ -11653,16 +11653,16 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="BG66" s="12">
-        <x:v>14</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="BH66" s="12" t="s">
-        <x:v>110</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="BI66" s="12">
-        <x:v>14</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="BJ66" s="12" t="s">
-        <x:v>135</x:v>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="67" spans="1:62">
@@ -11784,25 +11784,25 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="AN67" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AO67" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AP67" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ67" s="12">
         <x:v>55</x:v>
       </x:c>
       <x:c r="AR67" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AS67" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT67" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU67" s="12">
         <x:v>55</x:v>
@@ -11841,21 +11841,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG67" s="12">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="BH67" s="12" t="s">
-        <x:v>177</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="BI67" s="12">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="BJ67" s="12" t="s">
-        <x:v>177</x:v>
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:62">
       <x:c r="A68" s="11" t="s">
-        <x:v>178</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B68" s="12" t="s">
         <x:v>53</x:v>
@@ -11960,7 +11960,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="AJ68" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AK68" s="12" t="s">
         <x:v>55</x:v>
@@ -11975,10 +11975,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO68" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP68" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ68" s="12">
         <x:v>56</x:v>
@@ -11987,10 +11987,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS68" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT68" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU68" s="12">
         <x:v>56</x:v>
@@ -12008,7 +12008,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="AZ68" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BA68" s="12" t="s">
         <x:v>49</x:v>
@@ -12020,7 +12020,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="BD68" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE68" s="12" t="s">
         <x:v>49</x:v>
@@ -12032,18 +12032,18 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="BH68" s="12" t="s">
-        <x:v>112</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="BI68" s="12">
         <x:v>8</x:v>
       </x:c>
       <x:c r="BJ68" s="12" t="s">
-        <x:v>112</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:62">
       <x:c r="A69" s="11" t="s">
-        <x:v>179</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B69" s="12" t="s">
         <x:v>53</x:v>
@@ -12115,7 +12115,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="Y69" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="Z69" s="12" t="s">
         <x:v>49</x:v>
@@ -12163,10 +12163,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AO69" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP69" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ69" s="12">
         <x:v>57</x:v>
@@ -12175,10 +12175,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS69" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT69" s="12" t="s">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU69" s="12">
         <x:v>57</x:v>
@@ -12208,7 +12208,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="BD69" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BE69" s="12" t="s">
         <x:v>49</x:v>
@@ -12226,96 +12226,96 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="BJ69" s="12" t="s">
-        <x:v>146</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="70" spans="1:62">
       <x:c r="A70" s="13" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="B70" s="13" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="C70" s="7" t="s">
         <x:v>180</x:v>
-      </x:c>
-      <x:c r="B70" s="13" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="C70" s="7" t="s">
-        <x:v>181</x:v>
       </x:c>
       <x:c r="D70" s="7"/>
       <x:c r="E70" s="7"/>
       <x:c r="F70" s="7"/>
       <x:c r="G70" s="7" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="H70" s="7"/>
       <x:c r="I70" s="7"/>
       <x:c r="J70" s="7"/>
       <x:c r="K70" s="7" t="s">
-        <x:v>182</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="L70" s="7"/>
       <x:c r="M70" s="7"/>
       <x:c r="N70" s="7"/>
       <x:c r="O70" s="7" t="s">
-        <x:v>183</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="P70" s="7"/>
       <x:c r="Q70" s="7"/>
       <x:c r="R70" s="7"/>
       <x:c r="S70" s="7" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="T70" s="7"/>
       <x:c r="U70" s="7"/>
       <x:c r="V70" s="7"/>
       <x:c r="W70" s="7" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="X70" s="7"/>
       <x:c r="Y70" s="7"/>
       <x:c r="Z70" s="7"/>
       <x:c r="AA70" s="7" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="AB70" s="7"/>
       <x:c r="AC70" s="7"/>
       <x:c r="AD70" s="7"/>
       <x:c r="AE70" s="7" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="AF70" s="7"/>
       <x:c r="AG70" s="7"/>
       <x:c r="AH70" s="7"/>
       <x:c r="AI70" s="7" t="s">
-        <x:v>185</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="AJ70" s="7"/>
       <x:c r="AK70" s="7"/>
       <x:c r="AL70" s="7"/>
       <x:c r="AM70" s="7" t="s">
-        <x:v>183</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="AN70" s="7"/>
       <x:c r="AO70" s="7"/>
       <x:c r="AP70" s="7"/>
       <x:c r="AQ70" s="7" t="s">
-        <x:v>183</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="AR70" s="7"/>
       <x:c r="AS70" s="7"/>
       <x:c r="AT70" s="7"/>
       <x:c r="AU70" s="7" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="AV70" s="7"/>
       <x:c r="AW70" s="7"/>
       <x:c r="AX70" s="7"/>
       <x:c r="AY70" s="7" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="AZ70" s="7"/>
       <x:c r="BA70" s="7"/>
       <x:c r="BB70" s="7"/>
       <x:c r="BC70" s="7" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="BD70" s="7"/>
       <x:c r="BE70" s="7"/>

</xml_diff>